<commit_message>
docs: 공통 설계 규칙 created_at/updated_at/deleted_at 규칙을 DB 설계 리뷰 V2(2026-10-08) 기준으로 재정정 - created_at 전 테이블 필수 복원, updated_at 조건부 추가 규칙 명문화, deleted_at 판단 기준 추가
</commit_message>
<xml_diff>
--- a/docs/04_ERD_테이블정의서.xlsx
+++ b/docs/04_ERD_테이블정의서.xlsx
@@ -25643,22 +25643,26 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="59">
+    <row r="15" ht="27.75" customHeight="1" s="59">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  created_at / updated_at   필요한 테이블에만 선택적으로 추가 (전 테이블 일괄 적용 폐지 — 2026-10-08 팀 합의)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16.5" customHeight="1" s="59">
+          <t xml:space="preserve">  created_at   전 테이블 필수 — 목록 정렬·장애 추적에 공짜로 쓸모 있어 손해 없음. 타입 DATETIME, JPA는 BaseTimeEntity + Auditing으로 자동 처리 (2026-10-08 DB 설계 리뷰 V2 확정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="27.75" customHeight="1" s="59">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  → 추가할 경우 타입은 DATETIME. JPA는 BaseTimeEntity + @MappedSuperclass + Auditing 으로 자동 처리 가능</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="7.5" customHeight="1" s="59">
-      <c r="A17" s="13" t="n"/>
+          <t xml:space="preserve">  updated_at   조건부 — 로우 값이 생성 후에도 바뀔 수 있으면 추가. resolved_at/paid_at/used_at처럼 "무엇이 언제 바뀌었는지" 의미가 분명한 도메인 컬럼이 있으면 그쪽을 우선하고 generic updated_at은 생략 가능</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="27.75" customHeight="1" s="59">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  deleted_at   체크 하나 — "이 로우가 없어지면 다른 테이블의 참조가 깨지는가?" 로 판단. 삭제 기능이 없거나(로그성) 상태 필드로만 관리되는 테이블(거래 원장)에는 넣지 않음. UNIQUE 제약 걸린 단순 토글 테이블(likes 등)에는 오히려 넣지 않음</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="7.5" customHeight="1" s="59">
       <c r="A18" s="3" t="n"/>

</xml_diff>